<commit_message>
Se añadió la funcionalidad completa de Añadir Personaje y Eliminar Personaje, habiendo realizado pruebas de su funcionamiento. Se editó la API para añadir un nuevo método a HabilidadController para buscar habilidades por tipo, a su vez se editó la documentación y los diagramas de clases por dicho cambio.
</commit_message>
<xml_diff>
--- a/Planificación/to-do-list-proyecto.xlsx
+++ b/Planificación/to-do-list-proyecto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dynod\OneDrive\Escritorio\2º DAM - UNENDO\Proyecto Intermodular\Planificación\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dynod\OneDrive\Escritorio\2º DAM - UNENDO\Proyecto Intermodular\es_legacy_app_unendo_project\Planificación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A93845-05C5-45AF-8233-104BC6EC4584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BA5CEC-365E-4AE6-B320-D2404DDE1FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -909,7 +909,7 @@
       <c r="A37" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B37" s="3"/>
+      <c r="B37" s="4"/>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">

</xml_diff>

<commit_message>
Se añade la carpeta inicial base de la app móvil. Además de añadir la parte de financiación y costes en el documento, así como la imagen de las recompensas del crowdfunding. Esa parte ya está revisada y aprobada.
</commit_message>
<xml_diff>
--- a/Planificación/to-do-list-proyecto.xlsx
+++ b/Planificación/to-do-list-proyecto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dynod\OneDrive\Escritorio\2º DAM - UNENDO\Proyecto Intermodular\es_legacy_app_unendo_project\Planificación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BA5CEC-365E-4AE6-B320-D2404DDE1FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E40B06-459A-47CB-ABD0-25E9D68B7D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -166,7 +166,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -186,6 +186,13 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -319,7 +326,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -368,6 +374,7 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -682,66 +689,66 @@
         <v>26</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="12"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="11"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="18"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="17"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="4"/>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="20"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="E9" s="6" t="s">
+      <c r="B9" s="21"/>
+      <c r="E9" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -759,7 +766,7 @@
       <c r="A12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="5"/>
+      <c r="B12" s="4"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -885,7 +892,7 @@
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B33" s="3"/>
+      <c r="B33" s="4"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">

</xml_diff>

<commit_message>
Añadida la carpeta de la App de móvil con su versión mejorada, pero todavía pendiente de terminar. Se modificó el documento para añadir pruebas de integridad y algunas correcciones.
</commit_message>
<xml_diff>
--- a/Planificación/to-do-list-proyecto.xlsx
+++ b/Planificación/to-do-list-proyecto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dynod\OneDrive\Escritorio\2º DAM - UNENDO\Proyecto Intermodular\es_legacy_app_unendo_project\Planificación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E40B06-459A-47CB-ABD0-25E9D68B7D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051B5292-3CDE-407A-A422-67BC9CBA65B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -326,6 +326,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -374,7 +375,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -689,66 +689,66 @@
         <v>26</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="12"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="13"/>
-      <c r="G6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="15"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="16"/>
-      <c r="G7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="4"/>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="21"/>
-      <c r="E9" s="5" t="s">
+      <c r="B9" s="5"/>
+      <c r="E9" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="8"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -886,7 +886,7 @@
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="3"/>
+      <c r="B32" s="4"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
@@ -898,7 +898,7 @@
       <c r="A34" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B34" s="3"/>
+      <c r="B34" s="4"/>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">

</xml_diff>

<commit_message>
Se añadió el apartado de conclusiones al documento, y se generó el PDF provisional. A fecha de hoy queda en pendiente de revisión antes de la entrega final del proyecto.
</commit_message>
<xml_diff>
--- a/Planificación/to-do-list-proyecto.xlsx
+++ b/Planificación/to-do-list-proyecto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dynod\OneDrive\Escritorio\2º DAM - UNENDO\Proyecto Intermodular\es_legacy_app_unendo_project\Planificación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051B5292-3CDE-407A-A422-67BC9CBA65B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1333B57-5E56-4BF3-892C-FFB9DE6D75E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -318,13 +318,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -670,247 +669,247 @@
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="4"/>
+      <c r="B1" s="3"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4"/>
+      <c r="B2" s="3"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4"/>
+      <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="E4" s="9" t="s">
+      <c r="B4" s="3"/>
+      <c r="E4" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="E5" s="10" t="s">
+      <c r="B5" s="3"/>
+      <c r="E5" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="12"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="11"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="E6" s="13" t="s">
+      <c r="B6" s="3"/>
+      <c r="E6" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="E7" s="16" t="s">
+      <c r="B7" s="3"/>
+      <c r="E7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="18"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="17"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="E8" s="19" t="s">
+      <c r="B8" s="3"/>
+      <c r="E8" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="20"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="E9" s="6" t="s">
+      <c r="B9" s="4"/>
+      <c r="E9" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="4"/>
+      <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="4"/>
+      <c r="B11" s="3"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="4"/>
+      <c r="B12" s="3"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="4"/>
+      <c r="B13" s="3"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="4"/>
+      <c r="B14" s="3"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="4"/>
+      <c r="B15" s="3"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="4"/>
+      <c r="B16" s="3"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="4"/>
+      <c r="B17" s="3"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="4"/>
+      <c r="B18" s="3"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="4"/>
+      <c r="B19" s="3"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="4"/>
+      <c r="B20" s="3"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="4"/>
+      <c r="B21" s="3"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="4"/>
+      <c r="B22" s="3"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="4"/>
+      <c r="B23" s="3"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="4"/>
+      <c r="B24" s="3"/>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="4"/>
+      <c r="B25" s="3"/>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="4"/>
+      <c r="B26" s="3"/>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="4"/>
+      <c r="B27" s="3"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="4"/>
+      <c r="B28" s="3"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="4"/>
+      <c r="B29" s="3"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="4"/>
+      <c r="B30" s="3"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="4"/>
+      <c r="B31" s="3"/>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="4"/>
+      <c r="B32" s="3"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B33" s="4"/>
+      <c r="B33" s="3"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B34" s="4"/>
+      <c r="B34" s="3"/>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="3"/>
+      <c r="B35" s="4"/>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="3"/>
+      <c r="B36" s="4"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
@@ -922,13 +921,13 @@
       <c r="A38" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B38" s="3"/>
+      <c r="B38" s="4"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="3"/>
+      <c r="B39" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>